<commit_message>
fix: format deadlines for Korean review
</commit_message>
<xml_diff>
--- a/examples/sample-output.xlsx
+++ b/examples/sample-output.xlsx
@@ -61,7 +61,7 @@
     <t>서울특별시</t>
   </si>
   <si>
-    <t>2026-06-03T10:00:00</t>
+    <t>2026-06-03 오전 10:00</t>
   </si>
   <si>
     <t>건축공사업</t>
@@ -85,7 +85,7 @@
     <t>경기도</t>
   </si>
   <si>
-    <t>2026-06-01T14:00:00</t>
+    <t>2026-06-01 오후 2:00</t>
   </si>
   <si>
     <t>https://example.com/notices/20260500002</t>
@@ -106,7 +106,7 @@
     <t>인천광역시</t>
   </si>
   <si>
-    <t>2026-06-02T09:00:00</t>
+    <t>2026-06-02 오전 9:00</t>
   </si>
   <si>
     <t>전기안전관리</t>
@@ -130,7 +130,7 @@
     <t>부산광역시</t>
   </si>
   <si>
-    <t>2026-06-10T16:00:00</t>
+    <t>2026-06-10 오후 4:00</t>
   </si>
   <si>
     <t>https://example.com/notices/20260500004</t>
@@ -148,7 +148,7 @@
     <t>대전광역시</t>
   </si>
   <si>
-    <t>2026-05-31T11:00:00</t>
+    <t>2026-05-31 오전 11:00</t>
   </si>
   <si>
     <t>시설물유지관리업</t>
@@ -169,7 +169,7 @@
     <t>광주광역시</t>
   </si>
   <si>
-    <t>2026-06-07T10:00:00</t>
+    <t>2026-06-07 오전 10:00</t>
   </si>
   <si>
     <t>https://example.com/notices/20260500006</t>
@@ -187,7 +187,7 @@
     <t>대구광역시</t>
   </si>
   <si>
-    <t>2026-06-08T15:00:00</t>
+    <t>2026-06-08 오후 3:00</t>
   </si>
   <si>
     <t>엔지니어링사업</t>
@@ -208,7 +208,7 @@
     <t>울산광역시</t>
   </si>
   <si>
-    <t>2026-06-05T10:00:00</t>
+    <t>2026-06-05 오전 10:00</t>
   </si>
   <si>
     <t>전기공사업</t>
@@ -229,7 +229,7 @@
     <t>세종특별자치시</t>
   </si>
   <si>
-    <t>2026-06-04T13:00:00</t>
+    <t>2026-06-04 오후 1:00</t>
   </si>
   <si>
     <t>https://example.com/notices/20260500009</t>
@@ -247,7 +247,7 @@
     <t>강원특별자치도</t>
   </si>
   <si>
-    <t>2026-06-12T17:00:00</t>
+    <t>2026-06-12 오후 5:00</t>
   </si>
   <si>
     <t>공공시설관리</t>
@@ -268,7 +268,7 @@
     <t>충청북도</t>
   </si>
   <si>
-    <t>2026-06-15T10:00:00</t>
+    <t>2026-06-15 오전 10:00</t>
   </si>
   <si>
     <t>https://example.com/notices/20260500011</t>
@@ -286,7 +286,7 @@
     <t>충청남도</t>
   </si>
   <si>
-    <t>2026-05-30T10:00:00</t>
+    <t>2026-05-30 오전 10:00</t>
   </si>
   <si>
     <t>https://example.com/notices/20260500012</t>
@@ -304,7 +304,7 @@
     <t>전라북도</t>
   </si>
   <si>
-    <t>2026-06-20T11:00:00</t>
+    <t>2026-06-20 오전 11:00</t>
   </si>
   <si>
     <t>교통영향평가대행자</t>
@@ -325,7 +325,7 @@
     <t>전라남도</t>
   </si>
   <si>
-    <t>2026-06-18T14:00:00</t>
+    <t>2026-06-18 오후 2:00</t>
   </si>
   <si>
     <t>https://example.com/notices/20260500014</t>
@@ -343,7 +343,7 @@
     <t>경상북도</t>
   </si>
   <si>
-    <t>2026-06-06T10:00:00</t>
+    <t>2026-06-06 오전 10:00</t>
   </si>
   <si>
     <t>포장공사업</t>
@@ -364,7 +364,7 @@
     <t>경상남도</t>
   </si>
   <si>
-    <t>2026-06-09T10:00:00</t>
+    <t>2026-06-09 오전 10:00</t>
   </si>
   <si>
     <t>정보통신공사업</t>
@@ -385,7 +385,7 @@
     <t>제주특별자치도</t>
   </si>
   <si>
-    <t>2026-06-11T10:00:00</t>
+    <t>2026-06-11 오전 10:00</t>
   </si>
   <si>
     <t>안전진단전문기관</t>
@@ -403,7 +403,7 @@
     <t>OO면사무소</t>
   </si>
   <si>
-    <t>2026-05-29T10:00:00</t>
+    <t>2026-05-29 오전 10:00</t>
   </si>
   <si>
     <t>https://example.com/notices/20260500018</t>
@@ -418,7 +418,7 @@
     <t>OO교육청</t>
   </si>
   <si>
-    <t>2026-06-13T10:00:00</t>
+    <t>2026-06-13 오전 10:00</t>
   </si>
   <si>
     <t>https://example.com/notices/20260500019</t>
@@ -433,7 +433,7 @@
     <t>OO공원녹지사업소</t>
   </si>
   <si>
-    <t>2026-06-14T10:00:00</t>
+    <t>2026-06-14 오전 10:00</t>
   </si>
   <si>
     <t>조경식재공사업</t>
@@ -463,7 +463,7 @@
     <t>OO공공건축센터</t>
   </si>
   <si>
-    <t>2026-06-16T10:00:00</t>
+    <t>2026-06-16 오전 10:00</t>
   </si>
   <si>
     <t>건설엔지니어링업</t>

</xml_diff>

<commit_message>
fix: show Korean alerts and Nara notice links
</commit_message>
<xml_diff>
--- a/examples/sample-output.xlsx
+++ b/examples/sample-output.xlsx
@@ -31,9 +31,6 @@
     <t>기관명</t>
   </si>
   <si>
-    <t>지역</t>
-  </si>
-  <si>
     <t>예산</t>
   </si>
   <si>
@@ -58,13 +55,10 @@
     <t>OO교육지원청</t>
   </si>
   <si>
-    <t>서울특별시</t>
-  </si>
-  <si>
     <t>2026-06-03 오전 10:00</t>
   </si>
   <si>
-    <t>건축공사업</t>
+    <t>업종: 건축공사업</t>
   </si>
   <si>
     <t>https://example.com/notices/20260500001</t>
@@ -82,9 +76,6 @@
     <t>OO시청</t>
   </si>
   <si>
-    <t>경기도</t>
-  </si>
-  <si>
     <t>2026-06-01 오후 2:00</t>
   </si>
   <si>
@@ -103,13 +94,10 @@
     <t>OO시설관리공단</t>
   </si>
   <si>
-    <t>인천광역시</t>
-  </si>
-  <si>
     <t>2026-06-02 오전 9:00</t>
   </si>
   <si>
-    <t>전기안전관리</t>
+    <t>업종: 전기안전관리</t>
   </si>
   <si>
     <t>https://example.com/notices/20260500003</t>
@@ -127,9 +115,6 @@
     <t>OO정보산업진흥원</t>
   </si>
   <si>
-    <t>부산광역시</t>
-  </si>
-  <si>
     <t>2026-06-10 오후 4:00</t>
   </si>
   <si>
@@ -145,13 +130,10 @@
     <t>OO구청</t>
   </si>
   <si>
-    <t>대전광역시</t>
-  </si>
-  <si>
     <t>2026-05-31 오전 11:00</t>
   </si>
   <si>
-    <t>시설물유지관리업</t>
+    <t>업종: 시설물유지관리업</t>
   </si>
   <si>
     <t>https://example.com/notices/20260500005</t>
@@ -166,9 +148,6 @@
     <t>OO대학교</t>
   </si>
   <si>
-    <t>광주광역시</t>
-  </si>
-  <si>
     <t>2026-06-07 오전 10:00</t>
   </si>
   <si>
@@ -184,13 +163,10 @@
     <t>OO상하수도사업소</t>
   </si>
   <si>
-    <t>대구광역시</t>
-  </si>
-  <si>
     <t>2026-06-08 오후 3:00</t>
   </si>
   <si>
-    <t>엔지니어링사업</t>
+    <t>업종: 엔지니어링사업</t>
   </si>
   <si>
     <t>https://example.com/notices/20260500007</t>
@@ -205,13 +181,10 @@
     <t>OO문화재단</t>
   </si>
   <si>
-    <t>울산광역시</t>
-  </si>
-  <si>
     <t>2026-06-05 오전 10:00</t>
   </si>
   <si>
-    <t>전기공사업</t>
+    <t>업종: 전기공사업</t>
   </si>
   <si>
     <t>https://example.com/notices/20260500008</t>
@@ -226,9 +199,6 @@
     <t>OO고등학교</t>
   </si>
   <si>
-    <t>세종특별자치시</t>
-  </si>
-  <si>
     <t>2026-06-04 오후 1:00</t>
   </si>
   <si>
@@ -244,13 +214,10 @@
     <t>OO도시공사</t>
   </si>
   <si>
-    <t>강원특별자치도</t>
-  </si>
-  <si>
     <t>2026-06-12 오후 5:00</t>
   </si>
   <si>
-    <t>공공시설관리</t>
+    <t>업종: 공공시설관리</t>
   </si>
   <si>
     <t>https://example.com/notices/20260500010</t>
@@ -265,9 +232,6 @@
     <t>OO중학교</t>
   </si>
   <si>
-    <t>충청북도</t>
-  </si>
-  <si>
     <t>2026-06-15 오전 10:00</t>
   </si>
   <si>
@@ -283,9 +247,6 @@
     <t>OO군청</t>
   </si>
   <si>
-    <t>충청남도</t>
-  </si>
-  <si>
     <t>2026-05-30 오전 10:00</t>
   </si>
   <si>
@@ -301,13 +262,10 @@
     <t>OO개발공사</t>
   </si>
   <si>
-    <t>전라북도</t>
-  </si>
-  <si>
     <t>2026-06-20 오전 11:00</t>
   </si>
   <si>
-    <t>교통영향평가대행자</t>
+    <t>업종: 교통영향평가대행자</t>
   </si>
   <si>
     <t>https://example.com/notices/20260500013</t>
@@ -322,9 +280,6 @@
     <t>OO청년센터</t>
   </si>
   <si>
-    <t>전라남도</t>
-  </si>
-  <si>
     <t>2026-06-18 오후 2:00</t>
   </si>
   <si>
@@ -340,13 +295,10 @@
     <t>OO도로관리사업소</t>
   </si>
   <si>
-    <t>경상북도</t>
-  </si>
-  <si>
     <t>2026-06-06 오전 10:00</t>
   </si>
   <si>
-    <t>포장공사업</t>
+    <t>업종: 포장공사업</t>
   </si>
   <si>
     <t>https://example.com/notices/20260500015</t>
@@ -361,13 +313,10 @@
     <t>OO경찰서</t>
   </si>
   <si>
-    <t>경상남도</t>
-  </si>
-  <si>
     <t>2026-06-09 오전 10:00</t>
   </si>
   <si>
-    <t>정보통신공사업</t>
+    <t>업종: 정보통신공사업</t>
   </si>
   <si>
     <t>https://example.com/notices/20260500016</t>
@@ -382,13 +331,10 @@
     <t>OO안전센터</t>
   </si>
   <si>
-    <t>제주특별자치도</t>
-  </si>
-  <si>
     <t>2026-06-11 오전 10:00</t>
   </si>
   <si>
-    <t>안전진단전문기관</t>
+    <t>업종: 안전진단전문기관</t>
   </si>
   <si>
     <t>https://example.com/notices/20260500017</t>
@@ -436,7 +382,7 @@
     <t>2026-06-14 오전 10:00</t>
   </si>
   <si>
-    <t>조경식재공사업</t>
+    <t>업종: 조경식재공사업</t>
   </si>
   <si>
     <t>https://example.com/notices/20260500020</t>
@@ -466,7 +412,7 @@
     <t>2026-06-16 오전 10:00</t>
   </si>
   <si>
-    <t>건설엔지니어링업</t>
+    <t>업종: 건설엔지니어링업</t>
   </si>
   <si>
     <t>https://example.com/notices/20260500022</t>
@@ -531,11 +477,10 @@
     <col min="3" max="3" width="42" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="24" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="8" width="22" customWidth="1"/>
-    <col min="9" max="9" width="24" customWidth="1"/>
-    <col min="10" max="10" width="42" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="22" customWidth="1"/>
+    <col min="8" max="8" width="34" customWidth="1"/>
+    <col min="9" max="9" width="42" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -566,40 +511,34 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
         <v>10</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>12</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" s="2">
+        <v>1200000000</v>
+      </c>
+      <c r="G2" t="s">
         <v>13</v>
       </c>
-      <c r="F2" t="s">
+      <c r="H2" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="2">
-        <v>1200000000</v>
-      </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>15</v>
-      </c>
-      <c r="I2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J2" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="3">
@@ -607,28 +546,25 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" t="s">
         <v>18</v>
       </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
         <v>19</v>
       </c>
-      <c r="D3" t="s">
+      <c r="F3" s="2">
+        <v>85000000</v>
+      </c>
+      <c r="G3" t="s">
         <v>20</v>
       </c>
-      <c r="E3" t="s">
+      <c r="I3" t="s">
         <v>21</v>
-      </c>
-      <c r="F3" t="s">
-        <v>22</v>
-      </c>
-      <c r="G3" s="2">
-        <v>85000000</v>
-      </c>
-      <c r="H3" t="s">
-        <v>23</v>
-      </c>
-      <c r="J3" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="4">
@@ -636,31 +572,28 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" t="s">
         <v>25</v>
       </c>
-      <c r="C4" t="s">
+      <c r="F4" s="2">
+        <v>42000000</v>
+      </c>
+      <c r="G4" t="s">
         <v>26</v>
       </c>
-      <c r="D4" t="s">
+      <c r="H4" t="s">
         <v>27</v>
       </c>
-      <c r="E4" t="s">
+      <c r="I4" t="s">
         <v>28</v>
-      </c>
-      <c r="F4" t="s">
-        <v>29</v>
-      </c>
-      <c r="G4" s="2">
-        <v>42000000</v>
-      </c>
-      <c r="H4" t="s">
-        <v>30</v>
-      </c>
-      <c r="I4" t="s">
-        <v>31</v>
-      </c>
-      <c r="J4" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="5">
@@ -668,25 +601,22 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" t="s">
+        <v>32</v>
+      </c>
+      <c r="G5" t="s">
         <v>33</v>
       </c>
-      <c r="C5" t="s">
+      <c r="I5" t="s">
         <v>34</v>
-      </c>
-      <c r="D5" t="s">
-        <v>35</v>
-      </c>
-      <c r="E5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F5" t="s">
-        <v>37</v>
-      </c>
-      <c r="H5" t="s">
-        <v>38</v>
-      </c>
-      <c r="J5" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="6">
@@ -694,31 +624,28 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>37</v>
+      </c>
+      <c r="F6" s="2">
+        <v>210000000</v>
+      </c>
+      <c r="G6" t="s">
+        <v>38</v>
+      </c>
+      <c r="H6" t="s">
+        <v>39</v>
+      </c>
+      <c r="I6" t="s">
         <v>40</v>
-      </c>
-      <c r="C6" t="s">
-        <v>41</v>
-      </c>
-      <c r="D6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" t="s">
-        <v>42</v>
-      </c>
-      <c r="F6" t="s">
-        <v>43</v>
-      </c>
-      <c r="G6" s="2">
-        <v>210000000</v>
-      </c>
-      <c r="H6" t="s">
-        <v>44</v>
-      </c>
-      <c r="I6" t="s">
-        <v>45</v>
-      </c>
-      <c r="J6" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="7">
@@ -726,28 +653,25 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C7" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="D7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E7" t="s">
-        <v>49</v>
-      </c>
-      <c r="F7" t="s">
-        <v>50</v>
-      </c>
-      <c r="G7" s="2">
+        <v>43</v>
+      </c>
+      <c r="F7" s="2">
         <v>63000000</v>
       </c>
-      <c r="H7" t="s">
-        <v>51</v>
-      </c>
-      <c r="J7" t="s">
-        <v>52</v>
+      <c r="G7" t="s">
+        <v>44</v>
+      </c>
+      <c r="I7" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="8">
@@ -755,31 +679,28 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="C8" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="D8" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E8" t="s">
-        <v>55</v>
-      </c>
-      <c r="F8" t="s">
-        <v>56</v>
-      </c>
-      <c r="G8" s="2">
+        <v>48</v>
+      </c>
+      <c r="F8" s="2">
         <v>99000000</v>
       </c>
+      <c r="G8" t="s">
+        <v>49</v>
+      </c>
       <c r="H8" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="I8" t="s">
-        <v>58</v>
-      </c>
-      <c r="J8" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9">
@@ -787,31 +708,28 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="C9" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="D9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E9" t="s">
-        <v>62</v>
-      </c>
-      <c r="F9" t="s">
-        <v>63</v>
-      </c>
-      <c r="G9" s="2">
+        <v>54</v>
+      </c>
+      <c r="F9" s="2">
         <v>340000000</v>
       </c>
+      <c r="G9" t="s">
+        <v>55</v>
+      </c>
       <c r="H9" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="I9" t="s">
-        <v>65</v>
-      </c>
-      <c r="J9" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10">
@@ -819,28 +737,25 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="C10" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="D10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="E10" t="s">
-        <v>69</v>
-      </c>
-      <c r="F10" t="s">
-        <v>70</v>
-      </c>
-      <c r="G10" s="2">
+        <v>60</v>
+      </c>
+      <c r="F10" s="2">
         <v>18000000</v>
       </c>
-      <c r="H10" t="s">
-        <v>71</v>
-      </c>
-      <c r="J10" t="s">
-        <v>72</v>
+      <c r="G10" t="s">
+        <v>61</v>
+      </c>
+      <c r="I10" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="11">
@@ -848,31 +763,28 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="C11" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="D11" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E11" t="s">
-        <v>75</v>
-      </c>
-      <c r="F11" t="s">
-        <v>76</v>
-      </c>
-      <c r="G11" s="2">
+        <v>65</v>
+      </c>
+      <c r="F11" s="2">
         <v>150000000</v>
       </c>
+      <c r="G11" t="s">
+        <v>66</v>
+      </c>
       <c r="H11" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="I11" t="s">
-        <v>78</v>
-      </c>
-      <c r="J11" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
     </row>
     <row r="12">
@@ -880,31 +792,28 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="C12" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="D12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E12" t="s">
-        <v>82</v>
-      </c>
-      <c r="F12" t="s">
-        <v>83</v>
-      </c>
-      <c r="G12" s="2">
+        <v>71</v>
+      </c>
+      <c r="F12" s="2">
         <v>980000000</v>
       </c>
+      <c r="G12" t="s">
+        <v>72</v>
+      </c>
       <c r="H12" t="s">
-        <v>84</v>
+        <v>14</v>
       </c>
       <c r="I12" t="s">
-        <v>16</v>
-      </c>
-      <c r="J12" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13">
@@ -912,28 +821,25 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="C13" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="D13" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E13" t="s">
-        <v>88</v>
-      </c>
-      <c r="F13" t="s">
-        <v>89</v>
-      </c>
-      <c r="G13" s="2">
+        <v>76</v>
+      </c>
+      <c r="F13" s="2">
         <v>72000000</v>
       </c>
-      <c r="H13" t="s">
-        <v>90</v>
-      </c>
-      <c r="J13" t="s">
-        <v>91</v>
+      <c r="G13" t="s">
+        <v>77</v>
+      </c>
+      <c r="I13" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="14">
@@ -941,31 +847,28 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="C14" t="s">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="D14" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E14" t="s">
-        <v>94</v>
-      </c>
-      <c r="F14" t="s">
-        <v>95</v>
-      </c>
-      <c r="G14" s="2">
+        <v>81</v>
+      </c>
+      <c r="F14" s="2">
         <v>54000000</v>
       </c>
+      <c r="G14" t="s">
+        <v>82</v>
+      </c>
       <c r="H14" t="s">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="I14" t="s">
-        <v>97</v>
-      </c>
-      <c r="J14" t="s">
-        <v>98</v>
+        <v>84</v>
       </c>
     </row>
     <row r="15">
@@ -973,25 +876,22 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>99</v>
+        <v>85</v>
       </c>
       <c r="C15" t="s">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="D15" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="E15" t="s">
-        <v>101</v>
-      </c>
-      <c r="F15" t="s">
-        <v>102</v>
-      </c>
-      <c r="H15" t="s">
-        <v>103</v>
-      </c>
-      <c r="J15" t="s">
-        <v>104</v>
+        <v>87</v>
+      </c>
+      <c r="G15" t="s">
+        <v>88</v>
+      </c>
+      <c r="I15" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="16">
@@ -999,31 +899,28 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="C16" t="s">
-        <v>106</v>
+        <v>91</v>
       </c>
       <c r="D16" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E16" t="s">
-        <v>107</v>
-      </c>
-      <c r="F16" t="s">
-        <v>108</v>
-      </c>
-      <c r="G16" s="2">
+        <v>92</v>
+      </c>
+      <c r="F16" s="2">
         <v>450000000</v>
       </c>
+      <c r="G16" t="s">
+        <v>93</v>
+      </c>
       <c r="H16" t="s">
-        <v>109</v>
+        <v>94</v>
       </c>
       <c r="I16" t="s">
-        <v>110</v>
-      </c>
-      <c r="J16" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
     </row>
     <row r="17">
@@ -1031,31 +928,28 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>112</v>
+        <v>96</v>
       </c>
       <c r="C17" t="s">
-        <v>113</v>
+        <v>97</v>
       </c>
       <c r="D17" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E17" t="s">
-        <v>114</v>
-      </c>
-      <c r="F17" t="s">
-        <v>115</v>
-      </c>
-      <c r="G17" s="2">
+        <v>98</v>
+      </c>
+      <c r="F17" s="2">
         <v>115000000</v>
       </c>
+      <c r="G17" t="s">
+        <v>99</v>
+      </c>
       <c r="H17" t="s">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="I17" t="s">
-        <v>117</v>
-      </c>
-      <c r="J17" t="s">
-        <v>118</v>
+        <v>101</v>
       </c>
     </row>
     <row r="18">
@@ -1063,31 +957,28 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>119</v>
+        <v>102</v>
       </c>
       <c r="C18" t="s">
-        <v>120</v>
+        <v>103</v>
       </c>
       <c r="D18" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E18" t="s">
-        <v>121</v>
-      </c>
-      <c r="F18" t="s">
-        <v>122</v>
-      </c>
-      <c r="G18" s="2">
+        <v>104</v>
+      </c>
+      <c r="F18" s="2">
         <v>76000000</v>
       </c>
+      <c r="G18" t="s">
+        <v>105</v>
+      </c>
       <c r="H18" t="s">
-        <v>123</v>
+        <v>106</v>
       </c>
       <c r="I18" t="s">
-        <v>124</v>
-      </c>
-      <c r="J18" t="s">
-        <v>125</v>
+        <v>107</v>
       </c>
     </row>
     <row r="19">
@@ -1095,31 +986,28 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>126</v>
+        <v>108</v>
       </c>
       <c r="C19" t="s">
-        <v>127</v>
+        <v>109</v>
       </c>
       <c r="D19" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E19" t="s">
-        <v>128</v>
-      </c>
-      <c r="F19" t="s">
-        <v>22</v>
-      </c>
-      <c r="G19" s="2">
+        <v>110</v>
+      </c>
+      <c r="F19" s="2">
         <v>680000000</v>
       </c>
+      <c r="G19" t="s">
+        <v>111</v>
+      </c>
       <c r="H19" t="s">
-        <v>129</v>
+        <v>14</v>
       </c>
       <c r="I19" t="s">
-        <v>16</v>
-      </c>
-      <c r="J19" t="s">
-        <v>130</v>
+        <v>112</v>
       </c>
     </row>
     <row r="20">
@@ -1127,28 +1015,25 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>131</v>
+        <v>113</v>
       </c>
       <c r="C20" t="s">
-        <v>132</v>
+        <v>114</v>
       </c>
       <c r="D20" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E20" t="s">
-        <v>133</v>
-      </c>
-      <c r="F20" t="s">
-        <v>14</v>
-      </c>
-      <c r="G20" s="2">
+        <v>115</v>
+      </c>
+      <c r="F20" s="2">
         <v>132000000</v>
       </c>
-      <c r="H20" t="s">
-        <v>134</v>
-      </c>
-      <c r="J20" t="s">
-        <v>135</v>
+      <c r="G20" t="s">
+        <v>116</v>
+      </c>
+      <c r="I20" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="21">
@@ -1156,31 +1041,28 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="C21" t="s">
-        <v>137</v>
+        <v>119</v>
       </c>
       <c r="D21" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E21" t="s">
-        <v>138</v>
-      </c>
-      <c r="F21" t="s">
-        <v>37</v>
-      </c>
-      <c r="G21" s="2">
+        <v>120</v>
+      </c>
+      <c r="F21" s="2">
         <v>88000000</v>
       </c>
+      <c r="G21" t="s">
+        <v>121</v>
+      </c>
       <c r="H21" t="s">
-        <v>139</v>
+        <v>122</v>
       </c>
       <c r="I21" t="s">
-        <v>140</v>
-      </c>
-      <c r="J21" t="s">
-        <v>141</v>
+        <v>123</v>
       </c>
     </row>
     <row r="22">
@@ -1188,22 +1070,19 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>142</v>
+        <v>124</v>
       </c>
       <c r="C22" t="s">
-        <v>143</v>
+        <v>125</v>
       </c>
       <c r="D22" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="E22" t="s">
-        <v>144</v>
-      </c>
-      <c r="F22" t="s">
-        <v>43</v>
-      </c>
-      <c r="J22" t="s">
-        <v>145</v>
+        <v>126</v>
+      </c>
+      <c r="I22" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="23">
@@ -1211,34 +1090,31 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>146</v>
+        <v>128</v>
       </c>
       <c r="C23" t="s">
-        <v>147</v>
+        <v>129</v>
       </c>
       <c r="D23" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E23" t="s">
-        <v>148</v>
-      </c>
-      <c r="F23" t="s">
-        <v>29</v>
-      </c>
-      <c r="G23" s="2">
+        <v>130</v>
+      </c>
+      <c r="F23" s="2">
         <v>57000000</v>
       </c>
+      <c r="G23" t="s">
+        <v>131</v>
+      </c>
       <c r="H23" t="s">
-        <v>149</v>
+        <v>132</v>
       </c>
       <c r="I23" t="s">
-        <v>150</v>
-      </c>
-      <c r="J23" t="s">
-        <v>151</v>
+        <v>133</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J23"/>
+  <autoFilter ref="A1:I23"/>
 </worksheet>
 </file>
</xml_diff>